<commit_message>
Regenerate the example workbooks with cross-tab views
</commit_message>
<xml_diff>
--- a/ejemplos/resultados/horario-del-grupo.xlsx
+++ b/ejemplos/resultados/horario-del-grupo.xlsx
@@ -546,15 +546,15 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
       <c r="D4" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A4&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
     </row>
@@ -565,15 +565,15 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A5&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
     </row>
@@ -584,15 +584,15 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;B$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;C$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>IFERROR(INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0)),"")</f>
+        <f>IFERROR(IF(INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0))="","",INDEX(Casillas!$C$4:$C$12,MATCH($A6&amp;"|"&amp;D$3,Casillas!$H$4:$H$12,0))),"")</f>
         <v/>
       </c>
     </row>
@@ -619,7 +619,7 @@
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="37" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -667,7 +667,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>(clave)</t>
+          <t>(clave turno|dia)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the group timetable example workbook with an editable grid
</commit_message>
<xml_diff>
--- a/ejemplos/resultados/horario-del-grupo.xlsx
+++ b/ejemplos/resultados/horario-del-grupo.xlsx
@@ -498,7 +498,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="008EA9DB"/>
+    <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -546,17 +546,20 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="B4" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;B$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;B$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;B$3)*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="C4" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;C$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;C$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;C$3)*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="D4" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;D$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;D$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;D$3)*1,0),0))))</f>
-        <v/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -565,17 +568,20 @@
           <t>T2</t>
         </is>
       </c>
-      <c r="B5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;B$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;B$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;B$3)*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="C5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;C$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;C$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;C$3)*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="D5" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;D$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;D$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A5&amp;CHAR(31)&amp;D$3)*1,0),0))))</f>
-        <v/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -584,18 +590,13 @@
           <t>T3</t>
         </is>
       </c>
-      <c r="B6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;B$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;B$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;B$3)*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="C6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;C$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;C$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;C$3)*1,0),0))))</f>
-        <v/>
-      </c>
-      <c r="D6" s="3">
-        <f>IF(ISNA(MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;D$3)*1,0),0)),"",IF(ISBLANK(INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;D$3)*1,0),0))),"",INDEX('Casilla por casilla'!$C$4:$C$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A6&amp;CHAR(31)&amp;D$3)*1,0),0))))</f>
-        <v/>
-      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -610,6 +611,11 @@
       <formula>IFERROR(INDEX('Casilla por casilla'!$I$4:$I$12,MATCH(1,INDEX(EXACT('Casilla por casilla'!$J$4:$J$12,$A4&amp;CHAR(31)&amp;B$3)*1,0),0)),0)=1</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B4:D6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fuera del dominio" error="Ese valor no esta en la lista." type="list" errorStyle="information">
+      <formula1>'Listas'!$A$4:$A$7</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -707,10 +713,9 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
+      <c r="C4" s="3">
+        <f>IF(ISBLANK('Horario semanal'!B4),"",'Horario semanal'!B4)</f>
+        <v/>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -753,10 +758,9 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
+      <c r="C5" s="3">
+        <f>IF(ISBLANK('Horario semanal'!C4),"",'Horario semanal'!C4)</f>
+        <v/>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -799,10 +803,9 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
+      <c r="C6" s="3">
+        <f>IF(ISBLANK('Horario semanal'!D4),"",'Horario semanal'!D4)</f>
+        <v/>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -845,10 +848,9 @@
           <t>T2</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
+      <c r="C7" s="3">
+        <f>IF(ISBLANK('Horario semanal'!B5),"",'Horario semanal'!B5)</f>
+        <v/>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -891,10 +893,9 @@
           <t>T2</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>IP</t>
-        </is>
+      <c r="C8" s="3">
+        <f>IF(ISBLANK('Horario semanal'!C5),"",'Horario semanal'!C5)</f>
+        <v/>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -937,10 +938,9 @@
           <t>T2</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
+      <c r="C9" s="3">
+        <f>IF(ISBLANK('Horario semanal'!D5),"",'Horario semanal'!D5)</f>
+        <v/>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -983,7 +983,10 @@
           <t>T3</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n"/>
+      <c r="C10" s="3">
+        <f>IF(ISBLANK('Horario semanal'!B6),"",'Horario semanal'!B6)</f>
+        <v/>
+      </c>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Plan de la carrera'!$A$4:$A$7,$C10)*1,0),0)),"",IF(ISBLANK(INDEX('Plan de la carrera'!$B$4:$B$7,MATCH(1,INDEX(EXACT('Plan de la carrera'!$A$4:$A$7,$C10)*1,0),0))),"",INDEX('Plan de la carrera'!$B$4:$B$7,MATCH(1,INDEX(EXACT('Plan de la carrera'!$A$4:$A$7,$C10)*1,0),0))))</f>
@@ -1021,10 +1024,9 @@
           <t>T3</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
+      <c r="C11" s="3">
+        <f>IF(ISBLANK('Horario semanal'!C6),"",'Horario semanal'!C6)</f>
+        <v/>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -1067,7 +1069,10 @@
           <t>T3</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n"/>
+      <c r="C12" s="3">
+        <f>IF(ISBLANK('Horario semanal'!D6),"",'Horario semanal'!D6)</f>
+        <v/>
+      </c>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="3">
         <f>IF(ISNA(MATCH(1,INDEX(EXACT('Plan de la carrera'!$A$4:$A$7,$C12)*1,0),0)),"",IF(ISBLANK(INDEX('Plan de la carrera'!$B$4:$B$7,MATCH(1,INDEX(EXACT('Plan de la carrera'!$A$4:$A$7,$C12)*1,0),0))),"",INDEX('Plan de la carrera'!$B$4:$B$7,MATCH(1,INDEX(EXACT('Plan de la carrera'!$A$4:$A$7,$C12)*1,0),0))))</f>
@@ -1150,10 +1155,7 @@
       <formula>AND(NOT(($C4="")),(IFERROR(VALUE($G4&amp;""),0)&lt;0))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="C4:C12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fuera del dominio" error="Ese valor no esta en la lista." type="list" errorStyle="information">
-      <formula1>'Listas'!$A$4:$A$7</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="D4:D12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor fuera del dominio" error="Ese valor no esta en la lista." type="list" errorStyle="information">
       <formula1>'Listas'!$B$4:$B$6</formula1>
     </dataValidation>

</xml_diff>